<commit_message>
Update FPR/DS-020 R3 Future flows
</commit_message>
<xml_diff>
--- a/towers/FPR/DS Provide Decision Support/DS-020/input/data/R3_FutureFlows.xlsx
+++ b/towers/FPR/DS Provide Decision Support/DS-020/input/data/R3_FutureFlows.xlsx
@@ -1713,7 +1713,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="F30" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="G30" t="str">
         <v>Direct</v>
@@ -1751,7 +1751,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="D31" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="E31" t="str">
         <v>ECA-ADLS</v>
@@ -1933,7 +1933,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="F35" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="G35" t="str">
         <v>Direct</v>
@@ -1971,7 +1971,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="D36" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="E36" t="str">
         <v>ECA-ADLS</v>
@@ -2153,7 +2153,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="F40" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="G40" t="str">
         <v>Direct</v>
@@ -2191,7 +2191,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="D41" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="E41" t="str">
         <v>ECA-ADLS</v>
@@ -2373,7 +2373,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="F45" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="G45" t="str">
         <v>Direct</v>
@@ -2411,7 +2411,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="D46" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="E46" t="str">
         <v>ECA-ADLS</v>
@@ -2593,7 +2593,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="F50" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="G50" t="str">
         <v>Direct</v>
@@ -2631,7 +2631,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="D51" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="E51" t="str">
         <v>ECA-ADLS</v>
@@ -2813,7 +2813,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="F55" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="G55" t="str">
         <v>Direct</v>
@@ -2851,7 +2851,7 @@
         <v>Capacity Forecast Data Store</v>
       </c>
       <c r="D56" t="str">
-        <v>ECA Platform</v>
+        <v>Data Warehouse (IE)</v>
       </c>
       <c r="E56" t="str">
         <v>ECA-ADLS</v>

</xml_diff>